<commit_message>
ccreated a combined dataset spreadsheet
</commit_message>
<xml_diff>
--- a/dataset/01.w_Defects/dead_lock.xlsx
+++ b/dataset/01.w_Defects/dead_lock.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_002 () { pthread_t tid1; pthread_t tid2; pthread_t tid3; pthread_mutex_init(&amp;dead_lock_002_glb_mutexA, NULL); pthread_mutex_init(&amp;dead_lock_002_glb_mutexB, NULL); pthread_mutex_init(&amp;dead_lock_002_glb_mutexC, NULL); pthread_create(&amp;tid1, NULL, dead_lock_002_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_002_tsk_002, NULL); pthread_create(&amp;tid3, NULL, dead_lock_002_tsk_003, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_join(tid3, NULL); pthread_mutex_destroy(&amp;dead_lock_002_glb_mutexA); pthread_mutex_destroy(&amp;dead_lock_002_glb_mutexB); pthread_mutex_destroy(&amp;dead_lock_002_glb_mutexC); } void* dead_lock_002_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataB = (dead_lock_002_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexC); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataC = (dead_lock_002_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexC); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_002_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataA = (dead_lock_002_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataB = (dead_lock_002_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_002_tsk_003 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexC); /*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataC = (dead_lock_002_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataA = (dead_lock_002_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexC); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; }</t>
+          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_002 () { pthread_t tid1; pthread_t tid2; pthread_t tid3; pthread_mutex_init(&amp;dead_lock_002_glb_mutexA, NULL); pthread_mutex_init(&amp;dead_lock_002_glb_mutexB, NULL); pthread_mutex_init(&amp;dead_lock_002_glb_mutexC, NULL); pthread_create(&amp;tid1, NULL, dead_lock_002_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_002_tsk_002, NULL); pthread_create(&amp;tid3, NULL, dead_lock_002_tsk_003, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_join(tid3, NULL); pthread_mutex_destroy(&amp;dead_lock_002_glb_mutexA); pthread_mutex_destroy(&amp;dead_lock_002_glb_mutexB); pthread_mutex_destroy(&amp;dead_lock_002_glb_mutexC); } void* dead_lock_002_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataB = (dead_lock_002_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexC); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataC = (dead_lock_002_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexC); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_002_tsk_003 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexC); /*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataC = (dead_lock_002_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataA = (dead_lock_002_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexC); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_002_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataA = (dead_lock_002_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_002_glb_dataB = (dead_lock_002_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexB); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(&amp;dead_lock_002_glb_mutexA); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; }</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_003 () { pthread_t tid1; pthread_t tid2; pthread_mutex_init(dead_lock_003_glb_mutexA, NULL); pthread_mutex_init(dead_lock_003_glb_mutexB, NULL); pthread_mutex_init(dead_lock_003_glb_mutexC, NULL); pthread_create(&amp;tid1, NULL, dead_lock_003_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_003_tsk_002, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_mutex_destroy(dead_lock_003_glb_mutexA); pthread_mutex_destroy(dead_lock_003_glb_mutexB); pthread_mutex_destroy(dead_lock_003_glb_mutexC); } void* dead_lock_003_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataA = (dead_lock_003_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataB = (dead_lock_003_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataC = (dead_lock_003_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_003_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexB);/*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataB = (dead_lock_003_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataA = (dead_lock_003_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataC = (dead_lock_003_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; }</t>
+          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_003 () { pthread_t tid1; pthread_t tid2; pthread_mutex_init(dead_lock_003_glb_mutexA, NULL); pthread_mutex_init(dead_lock_003_glb_mutexB, NULL); pthread_mutex_init(dead_lock_003_glb_mutexC, NULL); pthread_create(&amp;tid1, NULL, dead_lock_003_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_003_tsk_002, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_mutex_destroy(dead_lock_003_glb_mutexA); pthread_mutex_destroy(dead_lock_003_glb_mutexB); pthread_mutex_destroy(dead_lock_003_glb_mutexC); } void* dead_lock_003_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexB);/*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataB = (dead_lock_003_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataA = (dead_lock_003_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataC = (dead_lock_003_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_003_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataA = (dead_lock_003_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataB = (dead_lock_003_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_003_glb_dataC = (dead_lock_003_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_003_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_003_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; }</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_004 () { pthread_t tid1; pthread_t tid2; pthread_mutex_init(dead_lock_004_glb_mutexA, NULL); pthread_mutex_init(dead_lock_004_glb_mutexB, NULL); pthread_mutex_init(dead_lock_004_glb_mutexC, NULL); pthread_create(&amp;tid1, NULL, dead_lock_004_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_004_tsk_002, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_mutex_destroy(dead_lock_004_glb_mutexA); pthread_mutex_destroy(dead_lock_004_glb_mutexB); pthread_mutex_destroy(dead_lock_004_glb_mutexC); } void* dead_lock_004_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataA = (dead_lock_004_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataB = (dead_lock_004_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataC = (dead_lock_004_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_004_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexB); /*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataB = (dead_lock_004_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataC = (dead_lock_004_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataA = (dead_lock_004_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; }</t>
+          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_004 () { pthread_t tid1; pthread_t tid2; pthread_mutex_init(dead_lock_004_glb_mutexA, NULL); pthread_mutex_init(dead_lock_004_glb_mutexB, NULL); pthread_mutex_init(dead_lock_004_glb_mutexC, NULL); pthread_create(&amp;tid1, NULL, dead_lock_004_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_004_tsk_002, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_mutex_destroy(dead_lock_004_glb_mutexA); pthread_mutex_destroy(dead_lock_004_glb_mutexB); pthread_mutex_destroy(dead_lock_004_glb_mutexC); } void* dead_lock_004_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexB); /*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataB = (dead_lock_004_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataC = (dead_lock_004_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataA = (dead_lock_004_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void* dead_lock_004_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataA = (dead_lock_004_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataB = (dead_lock_004_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_004_glb_dataC = (dead_lock_004_glb_dataC % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexC); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexC_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_004_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_004_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; }</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_005 () { printf("dead lock"); pthread_t tid1; pthread_t tid2; pthread_mutex_init(dead_lock_005_glb_mutexA, NULL); pthread_mutex_init(dead_lock_005_glb_mutexB, NULL); pthread_create(&amp;tid1, NULL, dead_lock_005_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_005_tsk_002, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_mutex_destroy(dead_lock_005_glb_mutexA); pthread_mutex_destroy(dead_lock_005_glb_mutexB); } void* dead_lock_005_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataA = (dead_lock_005_glb_dataA % 100) + 1; dead_lock_005_func_001(); #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void dead_lock_005_func_001 () { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataB = (dead_lock_005_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ } void* dead_lock_005_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataB = (dead_lock_005_glb_dataB % 100) + 1; dead_lock_005_func_002(); #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void dead_lock_005_func_002 () { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexA);/*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataA = (dead_lock_005_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ }</t>
+          <t>pthread_mutex_t dead_lock_001_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_001_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; int dead_lock_001_glb_dataA = 10; int dead_lock_001_glb_dataB = 10; pthread_mutex_t dead_lock_002_glb_mutexA = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexB = PTHREAD_MUTEX_INITIALIZER; pthread_mutex_t dead_lock_002_glb_mutexC = PTHREAD_MUTEX_INITIALIZER; int dead_lock_002_glb_dataA = 0; int dead_lock_002_glb_dataB = 0; int dead_lock_002_glb_dataC = 0; pthread_mutex_t dead_lock_003_glb_mutexA_; pthread_mutex_t dead_lock_003_glb_mutexB_; pthread_mutex_t dead_lock_003_glb_mutexC_; pthread_mutex_t *dead_lock_003_glb_mutexA = &amp;dead_lock_003_glb_mutexA_; pthread_mutex_t *dead_lock_003_glb_mutexB = &amp;dead_lock_003_glb_mutexB_; pthread_mutex_t *dead_lock_003_glb_mutexC = &amp;dead_lock_003_glb_mutexC_; int dead_lock_003_glb_dataA = 0; int dead_lock_003_glb_dataB = 0; int dead_lock_003_glb_dataC = 0; pthread_mutex_t dead_lock_004_glb_mutexA_; pthread_mutex_t dead_lock_004_glb_mutexB_; pthread_mutex_t dead_lock_004_glb_mutexC_; pthread_mutex_t *dead_lock_004_glb_mutexA = &amp;dead_lock_004_glb_mutexA_; pthread_mutex_t *dead_lock_004_glb_mutexB = &amp;dead_lock_004_glb_mutexB_; pthread_mutex_t *dead_lock_004_glb_mutexC = &amp;dead_lock_004_glb_mutexC_; int dead_lock_004_glb_dataA = 0; int dead_lock_004_glb_dataB = 0; int dead_lock_004_glb_dataC = 0; pthread_mutex_t dead_lock_005_glb_mutexA_; pthread_mutex_t dead_lock_005_glb_mutexB_; pthread_mutex_t *dead_lock_005_glb_mutexA = &amp;dead_lock_005_glb_mutexA_; pthread_mutex_t *dead_lock_005_glb_mutexB = &amp;dead_lock_005_glb_mutexB_; int dead_lock_005_glb_dataA = 0; int dead_lock_005_glb_dataB = 0; extern volatile int vflag; void dead_lock_005 () { printf("dead lock"); pthread_t tid1; pthread_t tid2; pthread_mutex_init(dead_lock_005_glb_mutexA, NULL); pthread_mutex_init(dead_lock_005_glb_mutexB, NULL); pthread_create(&amp;tid1, NULL, dead_lock_005_tsk_001, NULL); pthread_create(&amp;tid2, NULL, dead_lock_005_tsk_002, NULL); pthread_join(tid1, NULL); pthread_join(tid2, NULL); pthread_mutex_destroy(dead_lock_005_glb_mutexA); pthread_mutex_destroy(dead_lock_005_glb_mutexB); } void* dead_lock_005_tsk_002 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataB = (dead_lock_005_glb_dataB % 100) + 1; dead_lock_005_func_002(); #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void dead_lock_005_func_002 () { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexA);/*Tool should detect this line as error*/ /*ERROR:Dead Lock*/ #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataA = (dead_lock_005_glb_dataA % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ } void* dead_lock_005_tsk_001 (void *pram) { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataA = (dead_lock_005_glb_dataA % 100) + 1; dead_lock_005_func_001(); #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexA); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexA_); #endif /* ! defined(CHECKER_POLYSPACE) */ return NULL; } void dead_lock_005_func_001 () { #if ! defined(CHECKER_POLYSPACE) pthread_mutex_lock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_lock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ dead_lock_005_glb_dataB = (dead_lock_005_glb_dataB % 100) + 1; #if ! defined(CHECKER_POLYSPACE) pthread_mutex_unlock(dead_lock_005_glb_mutexB); #else /* ! defined(CHECKER_POLYSPACE) */ pthread_mutex_unlock(&amp;dead_lock_005_glb_mutexB_); #endif /* ! defined(CHECKER_POLYSPACE) */ }</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">

</xml_diff>